<commit_message>
Formation shift bug fixed.
</commit_message>
<xml_diff>
--- a/outputs/space-attack-prompts/prompts.xlsx
+++ b/outputs/space-attack-prompts/prompts.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompts" sheetId="1" r:id="Raa1e2c56e70c4e70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompts" sheetId="1" r:id="R0379f80184314020"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -387,6 +387,15 @@
         <x:v>Now let's add Wave tracking and initialization. When the last enemy on the screen has been removed, increment the wave counter by 1 and add a fresh grid of enemies to the board. The first wave of enemies should be a grid of 4 columns by 2 rows. With each additional wave, multiply the number of enemies by 1.2. Distribute enemies symmetrically across the center with a maximum grid width of 16 enemies and maximum of 6 rows. If a wave would exceed the maximum number of enemies, the Formation start speed is instead increased by x1.5. Also, if an enemy reaches the bottom of the canvas, deprecate the Lives by 1.</x:v>
       </x:c>
     </x:row>
+    <x:row r="10">
+      <x:c r="A10" s="12" t="n">
+        <x:v>46301.48673611111</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>there is currently a bug where, when an enemy is removed from a row, the other enemies in the row shift toward the center. When an enemy is removed via projectile hit, all remaining enemies in the grid should retain their placement. Same goes for upcoming advancing enemy state: if an enemy leaves the grid for any reason, the rest of the enemy formation grid should retain its position relative to the grid.
+Also, with each wave, let's increase the speed of the formation grid by 1.2, so that every wave is faster than the last one. Once the enemy grid is maximum size, then instead increase subsequent waves' starting speed by 1.5. Also, let's increase the formation grid direction speed change to 1.3 instead of 1.2.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Advancing behavior has been added for enemies.
</commit_message>
<xml_diff>
--- a/outputs/space-attack-prompts/prompts.xlsx
+++ b/outputs/space-attack-prompts/prompts.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompts" sheetId="1" r:id="R0379f80184314020"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompts" sheetId="1" r:id="R7237a0bb4ed34cc8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -396,6 +396,16 @@
 Also, with each wave, let's increase the speed of the formation grid by 1.2, so that every wave is faster than the last one. Once the enemy grid is maximum size, then instead increase subsequent waves' starting speed by 1.5. Also, let's increase the formation grid direction speed change to 1.3 instead of 1.2.</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" s="12" t="n">
+        <x:v>46301.494525462964</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>Double the delay for ship projectile firing. Change the increase in number of enemies per wave to a multiplier of 1.3.
+Let's now add an advancing state to the enemies. With each firing chance roll that currently occurs every 3 seconds, there is also a 0.1 chance that an enemy will shift into the advancing state.
+In the advancing state, the enemy will leave the group of enemies and begin a descending velocity of 1.4. It will fire a projectile every second while advancing. While advancing, the enemy's horizontal movement is bounded on the left and right sides by 248 points, unless the enemy hits the side of the canvas, at which point it will always change directions. The enemy should, when it goes into an advancing mode, leave the grid, descend toward the bottom of the screen while firing and drifting from left to right.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Change fonts and ship sprite to 8-bit style.
</commit_message>
<xml_diff>
--- a/outputs/space-attack-prompts/prompts.xlsx
+++ b/outputs/space-attack-prompts/prompts.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompts" sheetId="1" r:id="R7237a0bb4ed34cc8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompts" sheetId="1" r:id="R9c2bd2c87ca941f7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -406,6 +406,14 @@
 In the advancing state, the enemy will leave the group of enemies and begin a descending velocity of 1.4. It will fire a projectile every second while advancing. While advancing, the enemy's horizontal movement is bounded on the left and right sides by 248 points, unless the enemy hits the side of the canvas, at which point it will always change directions. The enemy should, when it goes into an advancing mode, leave the grid, descend toward the bottom of the screen while firing and drifting from left to right.</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="12" t="n">
+        <x:v>46301.50431712963</x:v>
+      </x:c>
+      <x:c r="B12" t="str">
+        <x:v>Change white text font size to 20 on the start state and the gameplay HUD.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Added screenshots and video recording
</commit_message>
<xml_diff>
--- a/outputs/space-attack-prompts/prompts.xlsx
+++ b/outputs/space-attack-prompts/prompts.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompts" sheetId="1" r:id="R9c2bd2c87ca941f7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Prompts" sheetId="1" r:id="R4723a5c28c1d4055"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -414,6 +414,14 @@
         <x:v>Change white text font size to 20 on the start state and the gameplay HUD.</x:v>
       </x:c>
     </x:row>
+    <x:row r="13">
+      <x:c r="A13" s="12" t="n">
+        <x:v>46301.50592592593</x:v>
+      </x:c>
+      <x:c r="B13" t="str">
+        <x:v>publish this site using Codex Sites</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>